<commit_message>
Created an new Scenario Configure course hierarchy pedagogy
</commit_message>
<xml_diff>
--- a/test-data/CourseData.xlsx
+++ b/test-data/CourseData.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t xml:space="preserve">DropdownIndex </t>
   </si>
@@ -41,6 +42,15 @@
   </si>
   <si>
     <t xml:space="preserve">Mern </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live Classes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Practical </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assesments </t>
   </si>
 </sst>
 </file>
@@ -50,11 +60,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -70,6 +81,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -119,12 +136,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -254,54 +283,54 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -314,4 +343,58 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.8"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
New Scenario added as Editing pedalogy
</commit_message>
<xml_diff>
--- a/test-data/CourseData.xlsx
+++ b/test-data/CourseData.xlsx
@@ -1,17 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LMS_PlayWright\test-data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC8F8A9C-B8D6-4F99-A383-D37486E64EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1"/>
@@ -21,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t xml:space="preserve">DropdownIndex </t>
   </si>
@@ -52,35 +58,32 @@
   <si>
     <t xml:space="preserve">Assesments </t>
   </si>
+  <si>
+    <t>skill</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>React</t>
+  </si>
+  <si>
+    <t>SQL</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="10"/>
@@ -103,7 +106,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -111,66 +114,37 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
@@ -212,14 +186,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -272,73 +246,71 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.18"/>
+    <col min="1" max="1" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
+    <row r="3" spans="1:2" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
+    <row r="5" spans="1:2" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
@@ -346,55 +318,86 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.8"/>
+    <col min="1" max="1" width="15.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667C45C1-39FE-4108-BDAE-2B154EB2CF88}">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add new Scenario Resource Type Adding
</commit_message>
<xml_diff>
--- a/test-data/CourseData.xlsx
+++ b/test-data/CourseData.xlsx
@@ -32,10 +32,10 @@
     <t xml:space="preserve">jamocha </t>
   </si>
   <si>
-    <t xml:space="preserve">Business to institution </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HTD </t>
+    <t xml:space="preserve">Automation Testing </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automation</t>
   </si>
   <si>
     <t xml:space="preserve">Software Development </t>
@@ -47,10 +47,10 @@
     <t xml:space="preserve">Live Classes </t>
   </si>
   <si>
-    <t xml:space="preserve">Practical </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assesments </t>
+    <t xml:space="preserve">cypress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assessment</t>
   </si>
 </sst>
 </file>
@@ -136,7 +136,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -149,11 +149,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -302,7 +306,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="23.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
@@ -318,7 +322,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
@@ -384,7 +388,7 @@
       <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
New Scenario added as Editing Resource Type
</commit_message>
<xml_diff>
--- a/test-data/CourseData.xlsx
+++ b/test-data/CourseData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LMS_PlayWright\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EE88A00-AF3C-4897-9FB1-4D56AE194812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E25E9A-C790-4F72-B825-7DE0438DC93F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="8880" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t xml:space="preserve">DropdownIndex </t>
   </si>
@@ -57,21 +57,6 @@
   </si>
   <si>
     <t xml:space="preserve">Assesments </t>
-  </si>
-  <si>
-    <t>skill</t>
-  </si>
-  <si>
-    <t>Python</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>React</t>
-  </si>
-  <si>
-    <t>SQL</t>
   </si>
 </sst>
 </file>
@@ -369,35 +354,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667C45C1-39FE-4108-BDAE-2B154EB2CF88}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Created an new Scenario E2E add course valid
</commit_message>
<xml_diff>
--- a/test-data/CourseData.xlsx
+++ b/test-data/CourseData.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t xml:space="preserve">DropdownIndex </t>
   </si>
@@ -51,6 +52,9 @@
   </si>
   <si>
     <t xml:space="preserve">Assessment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intermediate </t>
   </si>
 </sst>
 </file>
@@ -136,7 +140,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -158,6 +162,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -401,4 +409,39 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="23.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Data changed and error correction
</commit_message>
<xml_diff>
--- a/test-data/CourseData.xlsx
+++ b/test-data/CourseData.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
@@ -39,10 +39,10 @@
     <t xml:space="preserve">Tester </t>
   </si>
   <si>
-    <t xml:space="preserve">Software Development </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mern </t>
+    <t xml:space="preserve">software development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean Development</t>
   </si>
   <si>
     <t xml:space="preserve">Live Classes </t>
@@ -64,7 +64,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -92,11 +92,6 @@
       <family val="1"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -140,7 +135,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -150,10 +145,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -314,7 +305,7 @@
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -322,7 +313,7 @@
       <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -334,7 +325,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>4</v>
       </c>
@@ -376,7 +367,7 @@
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -384,7 +375,7 @@
       <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>8</v>
       </c>
     </row>
@@ -427,7 +418,7 @@
       <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>